<commit_message>
TICVAI r2: the HLD, LLD and AWS LLD regenerated at r2, so they name the DDoS protection CHG-R4-018 decided (build-hld-lld.py is not a refresh step); the mirrors follow
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/hld-lld/TICVAI - AWS Cloud Specs & Cost.xlsx
+++ b/ticvai/handoff/hld-lld/TICVAI - AWS Cloud Specs & Cost.xlsx
@@ -7070,12 +7070,12 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>Azure Front Door Premium + WAF (waiting-room page from cache)</t>
+          <t>Azure Front Door Premium + WAF (waiting-room page from cache; built-in DDoS protection)</t>
         </is>
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>Amazon CloudFront + AWS WAF (managed core rule set, Bot Control, rate-based rules); the waiting-room page from CloudFront's cache</t>
+          <t>Amazon CloudFront + AWS WAF (managed core rule set, Bot Control, rate-based rules); the waiting-room page from CloudFront's cache; AWS Shield Standard for DDoS</t>
         </is>
       </c>
     </row>

</xml_diff>